<commit_message>
added sign on box
</commit_message>
<xml_diff>
--- a/public/data/Master App Timesheet.xlsx
+++ b/public/data/Master App Timesheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\timesheet-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2CDAA7-1FB6-49B9-A870-21EE58EC147E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D26E902-3FCA-4E9C-8725-E8819756D339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vendor Entry Sheet" sheetId="5" r:id="rId1"/>
@@ -2961,6 +2961,123 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>57855</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>21166</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>275165</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>183443</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14DD9482-4B03-D611-85AE-5009589DAE86}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000" flipV="1">
+          <a:off x="3042355" y="7422444"/>
+          <a:ext cx="4937477" cy="2363610"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="1100" b="1"/>
+            <a:t>Greatland Supervisor Name:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="1100" b="1"/>
+            <a:t>Signiture</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="1100" b="1"/>
+            <a:t>Contractor Supervisor Name:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="1100" b="1"/>
+            <a:t>Signiture</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>228599</xdr:colOff>
       <xdr:row>1</xdr:row>
@@ -7091,6 +7208,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="89" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -30257,15 +30375,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="a1bbf4fc-2070-4842-8cf2-c42346818ea9" xsi:nil="true"/>
@@ -30274,6 +30383,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -30520,20 +30638,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71C3BF75-E265-495B-A1EF-9F0F8014FF62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C286B8F-44DD-46A1-8664-5B3AFC40D364}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="a1bbf4fc-2070-4842-8cf2-c42346818ea9"/>
     <ds:schemaRef ds:uri="d41b7399-51ed-4fce-9e89-79a41c55ed41"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71C3BF75-E265-495B-A1EF-9F0F8014FF62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>